<commit_message>
Added Squares and Tangent Values
</commit_message>
<xml_diff>
--- a/excel/flashcards_master.xlsx
+++ b/excel/flashcards_master.xlsx
@@ -5,19 +5,20 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrmath3/Documents/GitHub/mr-sindel-math/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrmath3/Documents/GitHub/Math-Flashcards/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42A9ABFE-341E-2C47-AEBF-DD0838AA60A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F1DA83C-24EF-1542-A3DD-41EDF101CDE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{DB8C5BD4-B13A-AA46-9C13-196CEA47E358}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="2" xr2:uid="{DB8C5BD4-B13A-AA46-9C13-196CEA47E358}"/>
   </bookViews>
   <sheets>
     <sheet name="cards_master" sheetId="1" r:id="rId1"/>
-    <sheet name="anki_export" sheetId="2" r:id="rId2"/>
-    <sheet name="blooket_export" sheetId="3" r:id="rId3"/>
-    <sheet name="quizlet_export" sheetId="4" r:id="rId4"/>
-    <sheet name="gimkit_export" sheetId="5" r:id="rId5"/>
+    <sheet name="export" sheetId="6" r:id="rId2"/>
+    <sheet name="anki" sheetId="2" r:id="rId3"/>
+    <sheet name="blooket" sheetId="3" r:id="rId4"/>
+    <sheet name="quizlet" sheetId="4" r:id="rId5"/>
+    <sheet name="gimkit" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,8 +40,45 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="170">
   <si>
     <t>deck</t>
   </si>
@@ -538,6 +576,18 @@
   </si>
   <si>
     <t>squares and square roots</t>
+  </si>
+  <si>
+    <t>Topic:</t>
+  </si>
+  <si>
+    <t>Tab:</t>
+  </si>
+  <si>
+    <t>squares_and_roots</t>
+  </si>
+  <si>
+    <t>anki</t>
   </si>
 </sst>
 </file>
@@ -603,6 +653,64 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>13</v>
+    <v>3</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="subType" t="i"/>
+  </s>
+</rvStructures>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2678,6 +2786,38 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0112EA51-173F-CF4F-8FFE-3FD34720780F}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="e" cm="1" vm="1">
+        <f t="array" ref="A4">_xlfn._xlws.FILTER(anki!A:C,(cards_master!B:B=B2))</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF2891CE-84D5-EF44-9F8F-0E7C3321DDFA}">
   <dimension ref="A1:C74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3865,7 +4005,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73CA60E6-D3E8-4544-887C-6E9318034364}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3874,7 +4014,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C35A34D1-7333-164B-A084-2BA53F3B571D}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3883,7 +4023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A4E6229-89EC-484C-B2E4-FE3173417D97}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>